<commit_message>
Refresh the Excel (capacity depth + Tetra Pak = cartons), dossier and PDF
Answers the founder's original question — the Excel now carries the
capacity-EXPANSION specifics, not just a headline:
- Roto Pack: the 42,000→57,540 MTPA path, the ~Rs430cr group capex, the
  14,600 MTPA Nath Foils plant (~40-50% used), and "no major new capex".
- GAEL: ~82% utilised, 5,000→6,000 TPD, the 850 TPD Hubli greenfield, the
  sodium-gluconate plant; Sayaji: single 950 TPD, no crush expansion.
- Chemco, PGP (1,730 TPD), Empire-Vitrum (single furnace) capacity added.
- Tetra Pak reclassified to "Aseptic cartons (NOT laminate film)".
- Triveni ownership corrected to Gerresheimer's 75% stake (not 100%).
- PDF rebuilt with this round's screenshots (% column, cartons category,
  Stock age tab, worst-terms-first credit) and the corrected dossier.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016cMuAas3DJJKm6WC5Hqjvx
</commit_message>
<xml_diff>
--- a/research/FDC-supplier-due-diligence.xlsx
+++ b/research/FDC-supplier-due-diligence.xlsx
@@ -144,7 +144,7 @@
     <t xml:space="preserve">Fortress: CARE/CRISIL AA-, effectively net-debt-free, ~₹950 cr cash. BUT profit is a commodity spread (one qtr -45%, then rebounded; FY26 PAT +22%).</t>
   </si>
   <si>
-    <t xml:space="preserve">5,000 TPD maize (#1 in India); ~₹600 cr capex; new fermentation (sodium gluconate) + pharma-grade starch line.</t>
+    <t xml:space="preserve">~5,000 TPD maize (#1 in India), ~82% utilised, expanding to 6,000 TPD; new 850 TPD greenfield at Hubli (Rs333cr, by FY2029); 30,000 TPA sodium-gluconate fermentation plant (commercial Dec-2025); dedicated food+pharma-grade starch capex via a WOS. Net-debt-free funding.</t>
   </si>
   <si>
     <t xml:space="preserve">2018 NGT pollution closure order at Sitarganj (stayed); minor GST demands. No fraud/insolvency.</t>
@@ -183,7 +183,7 @@
     <t xml:space="preserve">WAS DISTRESSED (FY25 operating profit negative; CARE BB+, below investment grade) — NOW RECOVERING (outlook moved to Positive, Sep-2026). Propped up by promoter loans + a ₹73 cr land sale.</t>
   </si>
   <si>
-    <t xml:space="preserve">950 TPD; NO real dextrose-capacity expansion planned (only automation capex).</t>
+    <t xml:space="preserve">Single 950 TPD plant (Kathwada, Ahmedabad; up from 930 TPD) — NO maize-crush expansion planned, only a ~Rs34cr automation/upgrade capex (FY27). Running near full, so it can take SOME extra volume, not a large block.</t>
   </si>
   <si>
     <t xml:space="preserve">A promoter dispute (Desai) settled 2021, no control change. No pollution/fire/recall found.</t>
@@ -219,7 +219,7 @@
     <t xml:space="preserve">~₹1,019 cr revenue (dipped FY24); CARE BBB+. BUT cash flow cratered ~80%, free cash ₹1.95 cr, high leverage (TD/GCA 10x).</t>
   </si>
   <si>
-    <t xml:space="preserve">57,540 MTPA across 2 Hyderabad plants (recently expanded). Live US exports.</t>
+    <t xml:space="preserve">57,540 MTPA laminate across 2 Hyderabad plants (Mankhal 28,200 + Burgul 29,340); grew from ~42,000 MTPA (FY22) via ~Rs430cr group capex (incl. a new 14,600 MTPA Nath Foils aluminium-foil plant at Aurangabad, commercial Mar-2024, only ~40-50% utilised). NO major new capex planned. Live US exports.</t>
   </si>
   <si>
     <t xml:space="preserve">No incidents/litigation found. India Ratings cut A-→BBB+ (Jan-2024) on leverage; CRISIL 'non-cooperating' (Aug-2024).</t>
@@ -264,7 +264,7 @@
     <t xml:space="preserve">CRISIL A+ / ICRA A+; revenue ₹602→939 cr in 3 yrs; gearing ~0.9x. Healthy.</t>
   </si>
   <si>
-    <t xml:space="preserve">&gt;125,000 t/yr across 23 locations + Gulf; built a &gt;1bn-bottle/yr food-grade rPET plant.</t>
+    <t xml:space="preserve">India's largest PET-preform maker (added &gt;25,000 t preform capacity in 2023 via 5 Husky lines); building an rPET pellet unit at Sanand (live ~Q3 FY26). Plenty of capacity + actively expanding. The ~125-day inventory is a deliberate model (CRISIL), not distress.</t>
   </si>
   <si>
     <t xml:space="preserve">No legal/pollution/fire/insolvency found. Absorbed Gaurav Containers (FY24).</t>
@@ -291,7 +291,7 @@
     <t xml:space="preserve">Tetra Pak India</t>
   </si>
   <si>
-    <t xml:space="preserve">Laminates (aseptic cartons)</t>
+    <t xml:space="preserve">Aseptic cartons (NOT laminate film)</t>
   </si>
   <si>
     <t xml:space="preserve">You pay too soon</t>
@@ -345,7 +345,7 @@
     <t xml:space="preserve">Heavily leveraged (combined gearing 5.64x); group did NOT cover interest in FY24 (0.86x); flagship revenue -23%. 'Rating-shopping' (2 agencies walked, a 3rd graded higher).</t>
   </si>
   <si>
-    <t xml:space="preserve">78,800 t/yr (~50% used — ample headroom).</t>
+    <t xml:space="preserve">Own flexible-laminate capacity (MTPA) NOT publicly disclosed by either rating agency; ~50% utilisation is the only headroom signal (Indian BOPET is in over-capacity). Capacity is not the concern here — the group's finances are.</t>
   </si>
   <si>
     <t xml:space="preserve">CAME WITHIN ONE COURT ORDER OF INSOLVENCY (NCLAT admitted 2025; Supreme Court reversed 2026). GROUP FATAL FIRE: a reactor blast at sister co GLS Speciality Chemicals killed 4 workers (May-2026); safety officer arrested; alleged ignored warnings.</t>
@@ -609,7 +609,7 @@
     <t xml:space="preserve">CRISIL A- / CARE A; cash-rich, low-geared (0.49x). FY26 PAT ~₹51 cr. Real-estate rentals are the group's profit engine (~60% margin).</t>
   </si>
   <si>
-    <t xml:space="preserve">Vikhroli plant; molded AMBER pharma glass (likely Type III, not confirmed Type I). ISO 9002.</t>
+    <t xml:space="preserve">Single Vikhroli (Mumbai) plant — ~1.9 million bottles/day (5-650 ml) of molded AMBER pharma glass; one furnace, so limited surge headroom. Likely Type III (Type I not confirmed). ISO 9002. Vitrum turnover ~Rs246cr.</t>
   </si>
   <si>
     <t xml:space="preserve">No pollution/fire/litigation found. A ₹33 cr doubtful-debt provision (possibly Gabon-linked) hit its trading arm.</t>
@@ -843,7 +843,7 @@
     <t xml:space="preserve">CARE A+; ~₹4,216 cr revenue, ~33% EBITDA margin, PAT ₹384 cr. A ₹2,597 cr ECB bullet due Mar-2026 being refinanced (Blackstone backstop).</t>
   </si>
   <si>
-    <t xml:space="preserve">~1,730 TPD, 12 furnaces; new Kosamba furnace (Jan-2025). Type I pharma-glass leader; global #1 in nail-polish bottles.</t>
+    <t xml:space="preserve">1,730 TPD glass (new 120 TPD Kosamba furnace added; up from 1,610); capex ~Rs600-700cr/yr FY26-27. Type I pharma-glass leader (pharma ~21% of sales); global #1 in nail-polish bottles. Ample capacity.</t>
   </si>
   <si>
     <t xml:space="preserve">Routine tax/excise disputes; a US product-liability suit. Zero fatalities FY25 (LTFIR rose). No pollution/recall found.</t>
@@ -915,7 +915,7 @@
     <t xml:space="preserve">The standout: a 'small' vendor that's actually a wholly-owned arm of GERRESHEIMER AG (German pharma-packaging MNC).</t>
   </si>
   <si>
-    <t xml:space="preserve">Private; 100% Gerresheimer AG (acquired 2012-18). Branded 'Gerresheimer Kundli'.</t>
+    <t xml:space="preserve">Private; Gerresheimer-controlled (took 75% in 2012; current exact stake not publicly confirmed). Branded 'Gerresheimer Kundli'.</t>
   </si>
   <si>
     <t xml:space="preserve">No free standalone financials, but MNC-backed and current on filings.</t>
@@ -1876,7 +1876,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
@@ -1929,7 +1929,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>48</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>61</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>73</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>103</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>189</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>268</v>
       </c>

</xml_diff>

<commit_message>
Founder feedback round: Tetra Pak cartons, deeper capacity research, % column, stock-age tab (#28)
Tetra Pak reclassified to its own "Aseptic cartons" category with the right (machine-compatible) carton peers; deep capacity/expansion/capex research folded into the plain-language supplier checks for all 27 with the "shift some, not all" framing and plant-proximity; a "% saved" column; a new "Stock age" tab; Credit & terms surfaces worst terms first so "100% advance" is visible; Triveni ownership corrected to Gerresheimer's 75% stake; Excel + PDF refreshed with the capacity depth.
</commit_message>
<xml_diff>
--- a/research/FDC-supplier-due-diligence.xlsx
+++ b/research/FDC-supplier-due-diligence.xlsx
@@ -144,7 +144,7 @@
     <t xml:space="preserve">Fortress: CARE/CRISIL AA-, effectively net-debt-free, ~₹950 cr cash. BUT profit is a commodity spread (one qtr -45%, then rebounded; FY26 PAT +22%).</t>
   </si>
   <si>
-    <t xml:space="preserve">5,000 TPD maize (#1 in India); ~₹600 cr capex; new fermentation (sodium gluconate) + pharma-grade starch line.</t>
+    <t xml:space="preserve">~5,000 TPD maize (#1 in India), ~82% utilised, expanding to 6,000 TPD; new 850 TPD greenfield at Hubli (Rs333cr, by FY2029); 30,000 TPA sodium-gluconate fermentation plant (commercial Dec-2025); dedicated food+pharma-grade starch capex via a WOS. Net-debt-free funding.</t>
   </si>
   <si>
     <t xml:space="preserve">2018 NGT pollution closure order at Sitarganj (stayed); minor GST demands. No fraud/insolvency.</t>
@@ -183,7 +183,7 @@
     <t xml:space="preserve">WAS DISTRESSED (FY25 operating profit negative; CARE BB+, below investment grade) — NOW RECOVERING (outlook moved to Positive, Sep-2026). Propped up by promoter loans + a ₹73 cr land sale.</t>
   </si>
   <si>
-    <t xml:space="preserve">950 TPD; NO real dextrose-capacity expansion planned (only automation capex).</t>
+    <t xml:space="preserve">Single 950 TPD plant (Kathwada, Ahmedabad; up from 930 TPD) — NO maize-crush expansion planned, only a ~Rs34cr automation/upgrade capex (FY27). Running near full, so it can take SOME extra volume, not a large block.</t>
   </si>
   <si>
     <t xml:space="preserve">A promoter dispute (Desai) settled 2021, no control change. No pollution/fire/recall found.</t>
@@ -219,7 +219,7 @@
     <t xml:space="preserve">~₹1,019 cr revenue (dipped FY24); CARE BBB+. BUT cash flow cratered ~80%, free cash ₹1.95 cr, high leverage (TD/GCA 10x).</t>
   </si>
   <si>
-    <t xml:space="preserve">57,540 MTPA across 2 Hyderabad plants (recently expanded). Live US exports.</t>
+    <t xml:space="preserve">57,540 MTPA laminate across 2 Hyderabad plants (Mankhal 28,200 + Burgul 29,340); grew from ~42,000 MTPA (FY22) via ~Rs430cr group capex (incl. a new 14,600 MTPA Nath Foils aluminium-foil plant at Aurangabad, commercial Mar-2024, only ~40-50% utilised). NO major new capex planned. Live US exports.</t>
   </si>
   <si>
     <t xml:space="preserve">No incidents/litigation found. India Ratings cut A-→BBB+ (Jan-2024) on leverage; CRISIL 'non-cooperating' (Aug-2024).</t>
@@ -264,7 +264,7 @@
     <t xml:space="preserve">CRISIL A+ / ICRA A+; revenue ₹602→939 cr in 3 yrs; gearing ~0.9x. Healthy.</t>
   </si>
   <si>
-    <t xml:space="preserve">&gt;125,000 t/yr across 23 locations + Gulf; built a &gt;1bn-bottle/yr food-grade rPET plant.</t>
+    <t xml:space="preserve">India's largest PET-preform maker (added &gt;25,000 t preform capacity in 2023 via 5 Husky lines); building an rPET pellet unit at Sanand (live ~Q3 FY26). Plenty of capacity + actively expanding. The ~125-day inventory is a deliberate model (CRISIL), not distress.</t>
   </si>
   <si>
     <t xml:space="preserve">No legal/pollution/fire/insolvency found. Absorbed Gaurav Containers (FY24).</t>
@@ -291,7 +291,7 @@
     <t xml:space="preserve">Tetra Pak India</t>
   </si>
   <si>
-    <t xml:space="preserve">Laminates (aseptic cartons)</t>
+    <t xml:space="preserve">Aseptic cartons (NOT laminate film)</t>
   </si>
   <si>
     <t xml:space="preserve">You pay too soon</t>
@@ -345,7 +345,7 @@
     <t xml:space="preserve">Heavily leveraged (combined gearing 5.64x); group did NOT cover interest in FY24 (0.86x); flagship revenue -23%. 'Rating-shopping' (2 agencies walked, a 3rd graded higher).</t>
   </si>
   <si>
-    <t xml:space="preserve">78,800 t/yr (~50% used — ample headroom).</t>
+    <t xml:space="preserve">Own flexible-laminate capacity (MTPA) NOT publicly disclosed by either rating agency; ~50% utilisation is the only headroom signal (Indian BOPET is in over-capacity). Capacity is not the concern here — the group's finances are.</t>
   </si>
   <si>
     <t xml:space="preserve">CAME WITHIN ONE COURT ORDER OF INSOLVENCY (NCLAT admitted 2025; Supreme Court reversed 2026). GROUP FATAL FIRE: a reactor blast at sister co GLS Speciality Chemicals killed 4 workers (May-2026); safety officer arrested; alleged ignored warnings.</t>
@@ -609,7 +609,7 @@
     <t xml:space="preserve">CRISIL A- / CARE A; cash-rich, low-geared (0.49x). FY26 PAT ~₹51 cr. Real-estate rentals are the group's profit engine (~60% margin).</t>
   </si>
   <si>
-    <t xml:space="preserve">Vikhroli plant; molded AMBER pharma glass (likely Type III, not confirmed Type I). ISO 9002.</t>
+    <t xml:space="preserve">Single Vikhroli (Mumbai) plant — ~1.9 million bottles/day (5-650 ml) of molded AMBER pharma glass; one furnace, so limited surge headroom. Likely Type III (Type I not confirmed). ISO 9002. Vitrum turnover ~Rs246cr.</t>
   </si>
   <si>
     <t xml:space="preserve">No pollution/fire/litigation found. A ₹33 cr doubtful-debt provision (possibly Gabon-linked) hit its trading arm.</t>
@@ -843,7 +843,7 @@
     <t xml:space="preserve">CARE A+; ~₹4,216 cr revenue, ~33% EBITDA margin, PAT ₹384 cr. A ₹2,597 cr ECB bullet due Mar-2026 being refinanced (Blackstone backstop).</t>
   </si>
   <si>
-    <t xml:space="preserve">~1,730 TPD, 12 furnaces; new Kosamba furnace (Jan-2025). Type I pharma-glass leader; global #1 in nail-polish bottles.</t>
+    <t xml:space="preserve">1,730 TPD glass (new 120 TPD Kosamba furnace added; up from 1,610); capex ~Rs600-700cr/yr FY26-27. Type I pharma-glass leader (pharma ~21% of sales); global #1 in nail-polish bottles. Ample capacity.</t>
   </si>
   <si>
     <t xml:space="preserve">Routine tax/excise disputes; a US product-liability suit. Zero fatalities FY25 (LTFIR rose). No pollution/recall found.</t>
@@ -915,7 +915,7 @@
     <t xml:space="preserve">The standout: a 'small' vendor that's actually a wholly-owned arm of GERRESHEIMER AG (German pharma-packaging MNC).</t>
   </si>
   <si>
-    <t xml:space="preserve">Private; 100% Gerresheimer AG (acquired 2012-18). Branded 'Gerresheimer Kundli'.</t>
+    <t xml:space="preserve">Private; Gerresheimer-controlled (took 75% in 2012; current exact stake not publicly confirmed). Branded 'Gerresheimer Kundli'.</t>
   </si>
   <si>
     <t xml:space="preserve">No free standalone financials, but MNC-backed and current on filings.</t>
@@ -1876,7 +1876,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
@@ -1929,7 +1929,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>48</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>61</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>73</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>103</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>189</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>268</v>
       </c>

</xml_diff>